<commit_message>
Subjects Json List Updated
</commit_message>
<xml_diff>
--- a/RESULTS/2017/CLASS/JSS1/FIRST/Mathematics/results.xlsx
+++ b/RESULTS/2017/CLASS/JSS1/FIRST/Mathematics/results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,118 +475,6 @@
       <c r="L1" t="inlineStr">
         <is>
           <t>Submitted At</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Abdulhakeem Maryam</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>std001</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>JSS1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>JSS1A</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>MATHEMATICS</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>FIRST</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>60</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>13</v>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>2026-08-20 11:09</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Ismail Ahmad Dikko</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>std002</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>JSS1</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>JSS1A</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>MATHEMATICS</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>FIRST</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>1%</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" t="n">
-        <v>60</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>FAIL</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>12</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>2026-08-20 11:10</t>
         </is>
       </c>
     </row>

</xml_diff>